<commit_message>
D3: extra rows allowed in the match rule; comparison rebuilt
On the 53 answerable queries the code system scores 47 vs ADAA 44;
overall 49 vs 49. Strict scores kept in extra columns.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/llm_codegen_experiment/results/comparison_adaa_vs_llm.xlsx
+++ b/llm_codegen_experiment/results/comparison_adaa_vs_llm.xlsx
@@ -12,7 +12,7 @@
     <sheet name="notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'comparison'!$A$1:$U$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'comparison'!$A$1:$W$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U64"/>
+  <dimension ref="A1:W64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -474,12 +474,14 @@
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="60" customWidth="1" min="14" max="14"/>
     <col width="60" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
     <col width="11" customWidth="1" min="21" max="21"/>
+    <col width="11" customWidth="1" min="22" max="22"/>
+    <col width="11" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -560,30 +562,40 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>adaa_extra_rows</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>llm_extra_rows</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>adaa_strict_match</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>llm_strict_match</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>adaa_cost_usd</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>llm_cost_usd</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>adaa_seconds</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>llm_seconds</t>
         </is>
@@ -649,22 +661,28 @@
       </c>
       <c r="N2" s="3" t="inlineStr"/>
       <c r="O2" s="3" t="inlineStr"/>
-      <c r="P2" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q2" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R2" s="2" t="n">
+      <c r="P2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T2" s="2" t="n">
         <v>0.000262</v>
       </c>
-      <c r="S2" s="2" t="n">
+      <c r="U2" s="2" t="n">
         <v>7.7e-05</v>
       </c>
-      <c r="T2" s="2" t="n">
+      <c r="V2" s="2" t="n">
         <v>2.44</v>
       </c>
-      <c r="U2" s="2" t="n">
+      <c r="W2" s="2" t="n">
         <v>2.18</v>
       </c>
     </row>
@@ -728,22 +746,28 @@
       </c>
       <c r="N3" s="3" t="inlineStr"/>
       <c r="O3" s="3" t="inlineStr"/>
-      <c r="P3" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q3" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R3" s="2" t="n">
+      <c r="P3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T3" s="2" t="n">
         <v>0.000263</v>
       </c>
-      <c r="S3" s="2" t="n">
+      <c r="U3" s="2" t="n">
         <v>7.9e-05</v>
       </c>
-      <c r="T3" s="2" t="n">
+      <c r="V3" s="2" t="n">
         <v>2.07</v>
       </c>
-      <c r="U3" s="2" t="n">
+      <c r="W3" s="2" t="n">
         <v>1.69</v>
       </c>
     </row>
@@ -807,22 +831,28 @@
       </c>
       <c r="N4" s="3" t="inlineStr"/>
       <c r="O4" s="3" t="inlineStr"/>
-      <c r="P4" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q4" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R4" s="2" t="n">
+      <c r="P4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T4" s="2" t="n">
         <v>0.000266</v>
       </c>
-      <c r="S4" s="2" t="n">
+      <c r="U4" s="2" t="n">
         <v>7.4e-05</v>
       </c>
-      <c r="T4" s="2" t="n">
+      <c r="V4" s="2" t="n">
         <v>1.85</v>
       </c>
-      <c r="U4" s="2" t="n">
+      <c r="W4" s="2" t="n">
         <v>1.58</v>
       </c>
     </row>
@@ -886,22 +916,28 @@
       </c>
       <c r="N5" s="3" t="inlineStr"/>
       <c r="O5" s="3" t="inlineStr"/>
-      <c r="P5" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q5" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R5" s="2" t="n">
+      <c r="P5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T5" s="2" t="n">
         <v>0.000262</v>
       </c>
-      <c r="S5" s="2" t="n">
+      <c r="U5" s="2" t="n">
         <v>7.6e-05</v>
       </c>
-      <c r="T5" s="2" t="n">
+      <c r="V5" s="2" t="n">
         <v>1.78</v>
       </c>
-      <c r="U5" s="2" t="n">
+      <c r="W5" s="2" t="n">
         <v>1.6</v>
       </c>
     </row>
@@ -965,22 +1001,28 @@
       </c>
       <c r="N6" s="3" t="inlineStr"/>
       <c r="O6" s="3" t="inlineStr"/>
-      <c r="P6" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q6" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R6" s="2" t="n">
+      <c r="P6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S6" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T6" s="2" t="n">
         <v>0.00026</v>
       </c>
-      <c r="S6" s="2" t="n">
+      <c r="U6" s="2" t="n">
         <v>8.1e-05</v>
       </c>
-      <c r="T6" s="2" t="n">
+      <c r="V6" s="2" t="n">
         <v>1.82</v>
       </c>
-      <c r="U6" s="2" t="n">
+      <c r="W6" s="2" t="n">
         <v>1.55</v>
       </c>
     </row>
@@ -1048,22 +1090,28 @@
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr"/>
-      <c r="P7" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R7" s="2" t="n">
+      <c r="P7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S7" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T7" s="2" t="n">
         <v>0.000261</v>
       </c>
-      <c r="S7" s="2" t="n">
+      <c r="U7" s="2" t="n">
         <v>8.000000000000001e-05</v>
       </c>
-      <c r="T7" s="2" t="n">
+      <c r="V7" s="2" t="n">
         <v>1.78</v>
       </c>
-      <c r="U7" s="2" t="n">
+      <c r="W7" s="2" t="n">
         <v>1.6</v>
       </c>
     </row>
@@ -1131,22 +1179,28 @@
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr"/>
-      <c r="P8" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R8" s="2" t="n">
+      <c r="P8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S8" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T8" s="2" t="n">
         <v>0.000257</v>
       </c>
-      <c r="S8" s="2" t="n">
+      <c r="U8" s="2" t="n">
         <v>8.000000000000001e-05</v>
       </c>
-      <c r="T8" s="2" t="n">
+      <c r="V8" s="2" t="n">
         <v>1.77</v>
       </c>
-      <c r="U8" s="2" t="n">
+      <c r="W8" s="2" t="n">
         <v>1.56</v>
       </c>
     </row>
@@ -1210,22 +1264,28 @@
       </c>
       <c r="N9" s="3" t="inlineStr"/>
       <c r="O9" s="3" t="inlineStr"/>
-      <c r="P9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R9" s="2" t="n">
+      <c r="P9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S9" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T9" s="2" t="n">
         <v>0.000295</v>
       </c>
-      <c r="S9" s="2" t="n">
+      <c r="U9" s="2" t="n">
         <v>8.1e-05</v>
       </c>
-      <c r="T9" s="2" t="n">
+      <c r="V9" s="2" t="n">
         <v>2.93</v>
       </c>
-      <c r="U9" s="2" t="n">
+      <c r="W9" s="2" t="n">
         <v>1.57</v>
       </c>
     </row>
@@ -1289,22 +1349,28 @@
       </c>
       <c r="N10" s="3" t="inlineStr"/>
       <c r="O10" s="3" t="inlineStr"/>
-      <c r="P10" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q10" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R10" s="2" t="n">
+      <c r="P10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T10" s="2" t="n">
         <v>0.000284</v>
       </c>
-      <c r="S10" s="2" t="n">
+      <c r="U10" s="2" t="n">
         <v>8.2e-05</v>
       </c>
-      <c r="T10" s="2" t="n">
+      <c r="V10" s="2" t="n">
         <v>2.81</v>
       </c>
-      <c r="U10" s="2" t="n">
+      <c r="W10" s="2" t="n">
         <v>1.58</v>
       </c>
     </row>
@@ -1368,22 +1434,28 @@
       </c>
       <c r="N11" s="3" t="inlineStr"/>
       <c r="O11" s="3" t="inlineStr"/>
-      <c r="P11" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q11" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R11" s="2" t="n">
+      <c r="P11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T11" s="2" t="n">
         <v>0.000286</v>
       </c>
-      <c r="S11" s="2" t="n">
+      <c r="U11" s="2" t="n">
         <v>8.000000000000001e-05</v>
       </c>
-      <c r="T11" s="2" t="n">
+      <c r="V11" s="2" t="n">
         <v>2.23</v>
       </c>
-      <c r="U11" s="2" t="n">
+      <c r="W11" s="2" t="n">
         <v>1.57</v>
       </c>
     </row>
@@ -1459,22 +1531,28 @@
       </c>
       <c r="N12" s="3" t="inlineStr"/>
       <c r="O12" s="3" t="inlineStr"/>
-      <c r="P12" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q12" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R12" s="2" t="n">
+      <c r="P12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S12" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T12" s="2" t="n">
         <v>0.000294</v>
       </c>
-      <c r="S12" s="2" t="n">
+      <c r="U12" s="2" t="n">
         <v>8.7e-05</v>
       </c>
-      <c r="T12" s="2" t="n">
+      <c r="V12" s="2" t="n">
         <v>2.47</v>
       </c>
-      <c r="U12" s="2" t="n">
+      <c r="W12" s="2" t="n">
         <v>2.24</v>
       </c>
     </row>
@@ -1550,22 +1628,28 @@
       </c>
       <c r="N13" s="3" t="inlineStr"/>
       <c r="O13" s="3" t="inlineStr"/>
-      <c r="P13" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q13" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R13" s="2" t="n">
+      <c r="P13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S13" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T13" s="2" t="n">
         <v>0.000306</v>
       </c>
-      <c r="S13" s="2" t="n">
+      <c r="U13" s="2" t="n">
         <v>9.7e-05</v>
       </c>
-      <c r="T13" s="2" t="n">
+      <c r="V13" s="2" t="n">
         <v>2.56</v>
       </c>
-      <c r="U13" s="2" t="n">
+      <c r="W13" s="2" t="n">
         <v>1.66</v>
       </c>
     </row>
@@ -1635,22 +1719,28 @@
       </c>
       <c r="N14" s="3" t="inlineStr"/>
       <c r="O14" s="3" t="inlineStr"/>
-      <c r="P14" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q14" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R14" s="2" t="n">
+      <c r="P14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S14" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T14" s="2" t="n">
         <v>0.000289</v>
       </c>
-      <c r="S14" s="2" t="n">
+      <c r="U14" s="2" t="n">
         <v>9.000000000000001e-05</v>
       </c>
-      <c r="T14" s="2" t="n">
+      <c r="V14" s="2" t="n">
         <v>2.49</v>
       </c>
-      <c r="U14" s="2" t="n">
+      <c r="W14" s="2" t="n">
         <v>1.64</v>
       </c>
     </row>
@@ -1729,22 +1819,28 @@
       </c>
       <c r="N15" s="3" t="inlineStr"/>
       <c r="O15" s="3" t="inlineStr"/>
-      <c r="P15" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q15" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R15" s="2" t="n">
+      <c r="P15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S15" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T15" s="2" t="n">
         <v>0.000328</v>
       </c>
-      <c r="S15" s="2" t="n">
+      <c r="U15" s="2" t="n">
         <v>9.000000000000001e-05</v>
       </c>
-      <c r="T15" s="2" t="n">
+      <c r="V15" s="2" t="n">
         <v>2.58</v>
       </c>
-      <c r="U15" s="2" t="n">
+      <c r="W15" s="2" t="n">
         <v>1.69</v>
       </c>
     </row>
@@ -1812,22 +1908,28 @@
           <t>wrong value: row 1: furniture, 0.1739226779820839 vs furniture</t>
         </is>
       </c>
-      <c r="P16" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q16" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R16" s="2" t="n">
+      <c r="P16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S16" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T16" s="2" t="n">
         <v>0.000292</v>
       </c>
-      <c r="S16" s="2" t="n">
+      <c r="U16" s="2" t="n">
         <v>8.7e-05</v>
       </c>
-      <c r="T16" s="2" t="n">
+      <c r="V16" s="2" t="n">
         <v>2.63</v>
       </c>
-      <c r="U16" s="2" t="n">
+      <c r="W16" s="2" t="n">
         <v>1.79</v>
       </c>
     </row>
@@ -1900,22 +2002,28 @@
       </c>
       <c r="N17" s="3" t="inlineStr"/>
       <c r="O17" s="3" t="inlineStr"/>
-      <c r="P17" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q17" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R17" s="2" t="n">
+      <c r="P17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S17" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T17" s="2" t="n">
         <v>0.000289</v>
       </c>
-      <c r="S17" s="2" t="n">
+      <c r="U17" s="2" t="n">
         <v>8.6e-05</v>
       </c>
-      <c r="T17" s="2" t="n">
+      <c r="V17" s="2" t="n">
         <v>3.36</v>
       </c>
-      <c r="U17" s="2" t="n">
+      <c r="W17" s="2" t="n">
         <v>1.55</v>
       </c>
     </row>
@@ -1983,22 +2091,28 @@
           <t>wrong value: row 1: november, 1471.0 vs 12.0, 1408.0</t>
         </is>
       </c>
-      <c r="P18" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q18" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R18" s="2" t="n">
+      <c r="P18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S18" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T18" s="2" t="n">
         <v>0.000303</v>
       </c>
-      <c r="S18" s="2" t="n">
+      <c r="U18" s="2" t="n">
         <v>0.000105</v>
       </c>
-      <c r="T18" s="2" t="n">
+      <c r="V18" s="2" t="n">
         <v>4.06</v>
       </c>
-      <c r="U18" s="2" t="n">
+      <c r="W18" s="2" t="n">
         <v>1.69</v>
       </c>
     </row>
@@ -2077,22 +2191,28 @@
           <t>wrong value: 16 rows returned, ground truth has 4</t>
         </is>
       </c>
-      <c r="P19" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q19" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R19" s="2" t="n">
+      <c r="P19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S19" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T19" s="2" t="n">
         <v>0.000294</v>
       </c>
-      <c r="S19" s="2" t="n">
+      <c r="U19" s="2" t="n">
         <v>9.500000000000001e-05</v>
       </c>
-      <c r="T19" s="2" t="n">
+      <c r="V19" s="2" t="n">
         <v>2.65</v>
       </c>
-      <c r="U19" s="2" t="n">
+      <c r="W19" s="2" t="n">
         <v>1.66</v>
       </c>
     </row>
@@ -2156,22 +2276,28 @@
       </c>
       <c r="N20" s="3" t="inlineStr"/>
       <c r="O20" s="3" t="inlineStr"/>
-      <c r="P20" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q20" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R20" s="2" t="n">
+      <c r="P20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S20" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T20" s="2" t="n">
         <v>0.000324</v>
       </c>
-      <c r="S20" s="2" t="n">
+      <c r="U20" s="2" t="n">
         <v>8.8e-05</v>
       </c>
-      <c r="T20" s="2" t="n">
+      <c r="V20" s="2" t="n">
         <v>4.07</v>
       </c>
-      <c r="U20" s="2" t="n">
+      <c r="W20" s="2" t="n">
         <v>1.74</v>
       </c>
     </row>
@@ -2235,22 +2361,28 @@
       </c>
       <c r="N21" s="3" t="inlineStr"/>
       <c r="O21" s="3" t="inlineStr"/>
-      <c r="P21" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q21" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R21" s="2" t="n">
+      <c r="P21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S21" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T21" s="2" t="n">
         <v>0.000295</v>
       </c>
-      <c r="S21" s="2" t="n">
+      <c r="U21" s="2" t="n">
         <v>9.8e-05</v>
       </c>
-      <c r="T21" s="2" t="n">
+      <c r="V21" s="2" t="n">
         <v>3.95</v>
       </c>
-      <c r="U21" s="2" t="n">
+      <c r="W21" s="2" t="n">
         <v>1.71</v>
       </c>
     </row>
@@ -2314,22 +2446,28 @@
       </c>
       <c r="N22" s="3" t="inlineStr"/>
       <c r="O22" s="3" t="inlineStr"/>
-      <c r="P22" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q22" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R22" s="2" t="n">
+      <c r="P22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S22" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T22" s="2" t="n">
         <v>0.000304</v>
       </c>
-      <c r="S22" s="2" t="n">
+      <c r="U22" s="2" t="n">
         <v>8.500000000000001e-05</v>
       </c>
-      <c r="T22" s="2" t="n">
+      <c r="V22" s="2" t="n">
         <v>3.02</v>
       </c>
-      <c r="U22" s="2" t="n">
+      <c r="W22" s="2" t="n">
         <v>1.58</v>
       </c>
     </row>
@@ -2397,22 +2535,28 @@
           <t>[error] error: TypeError: int() argument must be a string, a bytes-like object or a real number, not 'Series'</t>
         </is>
       </c>
-      <c r="P23" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q23" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R23" s="2" t="n">
+      <c r="P23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S23" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T23" s="2" t="n">
         <v>0.000311</v>
       </c>
-      <c r="S23" s="2" t="n">
+      <c r="U23" s="2" t="n">
         <v>0.000101</v>
       </c>
-      <c r="T23" s="2" t="n">
+      <c r="V23" s="2" t="n">
         <v>3.13</v>
       </c>
-      <c r="U23" s="2" t="n">
+      <c r="W23" s="2" t="n">
         <v>1.7</v>
       </c>
     </row>
@@ -2476,22 +2620,28 @@
       </c>
       <c r="N24" s="3" t="inlineStr"/>
       <c r="O24" s="3" t="inlineStr"/>
-      <c r="P24" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q24" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R24" s="2" t="n">
+      <c r="P24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S24" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T24" s="2" t="n">
         <v>0.000437</v>
       </c>
-      <c r="S24" s="2" t="n">
+      <c r="U24" s="2" t="n">
         <v>9.000000000000001e-05</v>
       </c>
-      <c r="T24" s="2" t="n">
+      <c r="V24" s="2" t="n">
         <v>4.5</v>
       </c>
-      <c r="U24" s="2" t="n">
+      <c r="W24" s="2" t="n">
         <v>2.03</v>
       </c>
     </row>
@@ -2555,22 +2705,28 @@
       </c>
       <c r="N25" s="3" t="inlineStr"/>
       <c r="O25" s="3" t="inlineStr"/>
-      <c r="P25" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q25" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R25" s="2" t="n">
+      <c r="P25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S25" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T25" s="2" t="n">
         <v>0.0003</v>
       </c>
-      <c r="S25" s="2" t="n">
+      <c r="U25" s="2" t="n">
         <v>8.8e-05</v>
       </c>
-      <c r="T25" s="2" t="n">
+      <c r="V25" s="2" t="n">
         <v>3.53</v>
       </c>
-      <c r="U25" s="2" t="n">
+      <c r="W25" s="2" t="n">
         <v>1.71</v>
       </c>
     </row>
@@ -2646,22 +2802,28 @@
       </c>
       <c r="N26" s="3" t="inlineStr"/>
       <c r="O26" s="3" t="inlineStr"/>
-      <c r="P26" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q26" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R26" s="2" t="n">
+      <c r="P26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S26" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T26" s="2" t="n">
         <v>0.000316</v>
       </c>
-      <c r="S26" s="2" t="n">
+      <c r="U26" s="2" t="n">
         <v>9.8e-05</v>
       </c>
-      <c r="T26" s="2" t="n">
+      <c r="V26" s="2" t="n">
         <v>3.77</v>
       </c>
-      <c r="U26" s="2" t="n">
+      <c r="W26" s="2" t="n">
         <v>1.74</v>
       </c>
     </row>
@@ -2725,22 +2887,28 @@
       </c>
       <c r="N27" s="3" t="inlineStr"/>
       <c r="O27" s="3" t="inlineStr"/>
-      <c r="P27" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q27" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R27" s="2" t="n">
+      <c r="P27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S27" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T27" s="2" t="n">
         <v>0.00029</v>
       </c>
-      <c r="S27" s="2" t="n">
+      <c r="U27" s="2" t="n">
         <v>8.4e-05</v>
       </c>
-      <c r="T27" s="2" t="n">
+      <c r="V27" s="2" t="n">
         <v>3.06</v>
       </c>
-      <c r="U27" s="2" t="n">
+      <c r="W27" s="2" t="n">
         <v>1.67</v>
       </c>
     </row>
@@ -2785,8 +2953,8 @@
       <c r="H28" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="I28" s="5" t="b">
-        <v>0</v>
+      <c r="I28" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
@@ -2795,7 +2963,7 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>wrong_answer</t>
+          <t>correct</t>
         </is>
       </c>
       <c r="L28" s="2" t="b">
@@ -2805,27 +2973,29 @@
         <v>0</v>
       </c>
       <c r="N28" s="3" t="inlineStr"/>
-      <c r="O28" s="3" t="inlineStr">
-        <is>
-          <t>wrong value: 3 rows returned, ground truth has 1</t>
-        </is>
-      </c>
-      <c r="P28" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q28" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R28" s="2" t="n">
+      <c r="O28" s="3" t="inlineStr"/>
+      <c r="P28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="R28" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S28" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T28" s="2" t="n">
         <v>0.000321</v>
       </c>
-      <c r="S28" s="2" t="n">
+      <c r="U28" s="2" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T28" s="2" t="n">
+      <c r="V28" s="2" t="n">
         <v>3.72</v>
       </c>
-      <c r="U28" s="2" t="n">
+      <c r="W28" s="2" t="n">
         <v>1.82</v>
       </c>
     </row>
@@ -2871,8 +3041,8 @@
       <c r="H29" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="I29" s="5" t="b">
-        <v>0</v>
+      <c r="I29" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
@@ -2881,7 +3051,7 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>wrong_answer</t>
+          <t>correct</t>
         </is>
       </c>
       <c r="L29" s="2" t="b">
@@ -2891,27 +3061,29 @@
         <v>0</v>
       </c>
       <c r="N29" s="3" t="inlineStr"/>
-      <c r="O29" s="3" t="inlineStr">
-        <is>
-          <t>wrong value: 4 rows returned, ground truth has 1</t>
-        </is>
-      </c>
-      <c r="P29" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q29" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R29" s="2" t="n">
+      <c r="O29" s="3" t="inlineStr"/>
+      <c r="P29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="R29" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S29" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T29" s="2" t="n">
         <v>0.000305</v>
       </c>
-      <c r="S29" s="2" t="n">
+      <c r="U29" s="2" t="n">
         <v>0.000107</v>
       </c>
-      <c r="T29" s="2" t="n">
+      <c r="V29" s="2" t="n">
         <v>4.06</v>
       </c>
-      <c r="U29" s="2" t="n">
+      <c r="W29" s="2" t="n">
         <v>1.67</v>
       </c>
     </row>
@@ -2975,22 +3147,28 @@
       </c>
       <c r="N30" s="3" t="inlineStr"/>
       <c r="O30" s="3" t="inlineStr"/>
-      <c r="P30" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q30" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R30" s="2" t="n">
+      <c r="P30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R30" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S30" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T30" s="2" t="n">
         <v>0.000312</v>
       </c>
-      <c r="S30" s="2" t="n">
+      <c r="U30" s="2" t="n">
         <v>9.1e-05</v>
       </c>
-      <c r="T30" s="2" t="n">
+      <c r="V30" s="2" t="n">
         <v>3.42</v>
       </c>
-      <c r="U30" s="2" t="n">
+      <c r="W30" s="2" t="n">
         <v>1.75</v>
       </c>
     </row>
@@ -3066,22 +3244,28 @@
       </c>
       <c r="N31" s="3" t="inlineStr"/>
       <c r="O31" s="3" t="inlineStr"/>
-      <c r="P31" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q31" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R31" s="2" t="n">
+      <c r="P31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S31" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T31" s="2" t="n">
         <v>0.000324</v>
       </c>
-      <c r="S31" s="2" t="n">
+      <c r="U31" s="2" t="n">
         <v>0.000111</v>
       </c>
-      <c r="T31" s="2" t="n">
+      <c r="V31" s="2" t="n">
         <v>3.87</v>
       </c>
-      <c r="U31" s="2" t="n">
+      <c r="W31" s="2" t="n">
         <v>1.67</v>
       </c>
     </row>
@@ -3134,8 +3318,8 @@
       <c r="H32" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="I32" s="5" t="b">
-        <v>0</v>
+      <c r="I32" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
@@ -3144,7 +3328,7 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>wrong_answer</t>
+          <t>correct</t>
         </is>
       </c>
       <c r="L32" s="2" t="b">
@@ -3154,27 +3338,29 @@
         <v>0</v>
       </c>
       <c r="N32" s="3" t="inlineStr"/>
-      <c r="O32" s="3" t="inlineStr">
-        <is>
-          <t>wrong value: 5 rows returned, ground truth has 4</t>
-        </is>
-      </c>
-      <c r="P32" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q32" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R32" s="2" t="n">
+      <c r="O32" s="3" t="inlineStr"/>
+      <c r="P32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R32" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S32" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T32" s="2" t="n">
         <v>0.000319</v>
       </c>
-      <c r="S32" s="2" t="n">
+      <c r="U32" s="2" t="n">
         <v>0.000112</v>
       </c>
-      <c r="T32" s="2" t="n">
+      <c r="V32" s="2" t="n">
         <v>1.9</v>
       </c>
-      <c r="U32" s="2" t="n">
+      <c r="W32" s="2" t="n">
         <v>2.24</v>
       </c>
     </row>
@@ -3224,8 +3410,8 @@
       <c r="H33" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="I33" s="5" t="b">
-        <v>0</v>
+      <c r="I33" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
@@ -3234,7 +3420,7 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>wrong_answer</t>
+          <t>correct</t>
         </is>
       </c>
       <c r="L33" s="2" t="b">
@@ -3244,27 +3430,29 @@
         <v>0</v>
       </c>
       <c r="N33" s="3" t="inlineStr"/>
-      <c r="O33" s="3" t="inlineStr">
-        <is>
-          <t>wrong value: 4 rows returned, ground truth has 3</t>
-        </is>
-      </c>
-      <c r="P33" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q33" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R33" s="2" t="n">
+      <c r="O33" s="3" t="inlineStr"/>
+      <c r="P33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R33" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S33" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T33" s="2" t="n">
         <v>0.000322</v>
       </c>
-      <c r="S33" s="2" t="n">
+      <c r="U33" s="2" t="n">
         <v>0.000106</v>
       </c>
-      <c r="T33" s="2" t="n">
+      <c r="V33" s="2" t="n">
         <v>1.8</v>
       </c>
-      <c r="U33" s="2" t="n">
+      <c r="W33" s="2" t="n">
         <v>2.18</v>
       </c>
     </row>
@@ -3312,8 +3500,8 @@
       <c r="H34" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="I34" s="5" t="b">
-        <v>0</v>
+      <c r="I34" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
@@ -3322,7 +3510,7 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>wrong_answer</t>
+          <t>correct</t>
         </is>
       </c>
       <c r="L34" s="2" t="b">
@@ -3336,27 +3524,29 @@
           <t>Planner: refused an answerable query | refused an answerable query: Query cannot be answered with available tools: The query requests both an overall average and a per-category average. According to the rules</t>
         </is>
       </c>
-      <c r="O34" s="3" t="inlineStr">
-        <is>
-          <t>wrong value: 4 rows returned, ground truth has 3</t>
-        </is>
-      </c>
-      <c r="P34" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q34" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R34" s="2" t="n">
+      <c r="O34" s="3" t="inlineStr"/>
+      <c r="P34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R34" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S34" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T34" s="2" t="n">
         <v>0.000341</v>
       </c>
-      <c r="S34" s="2" t="n">
+      <c r="U34" s="2" t="n">
         <v>0.000102</v>
       </c>
-      <c r="T34" s="2" t="n">
+      <c r="V34" s="2" t="n">
         <v>1.52</v>
       </c>
-      <c r="U34" s="2" t="n">
+      <c r="W34" s="2" t="n">
         <v>1.59</v>
       </c>
     </row>
@@ -3409,8 +3599,8 @@
       <c r="H35" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="I35" s="5" t="b">
-        <v>0</v>
+      <c r="I35" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
@@ -3419,7 +3609,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>wrong_answer</t>
+          <t>correct</t>
         </is>
       </c>
       <c r="L35" s="2" t="b">
@@ -3429,27 +3619,29 @@
         <v>0</v>
       </c>
       <c r="N35" s="3" t="inlineStr"/>
-      <c r="O35" s="3" t="inlineStr">
-        <is>
-          <t>wrong value: 5 rows returned, ground truth has 4</t>
-        </is>
-      </c>
-      <c r="P35" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q35" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R35" s="2" t="n">
+      <c r="O35" s="3" t="inlineStr"/>
+      <c r="P35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R35" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S35" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T35" s="2" t="n">
         <v>0.000363</v>
       </c>
-      <c r="S35" s="2" t="n">
+      <c r="U35" s="2" t="n">
         <v>0.000131</v>
       </c>
-      <c r="T35" s="2" t="n">
+      <c r="V35" s="2" t="n">
         <v>3.59</v>
       </c>
-      <c r="U35" s="2" t="n">
+      <c r="W35" s="2" t="n">
         <v>2.05</v>
       </c>
     </row>
@@ -3502,8 +3694,8 @@
       <c r="H36" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="I36" s="5" t="b">
-        <v>0</v>
+      <c r="I36" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
@@ -3512,7 +3704,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>wrong_answer</t>
+          <t>correct</t>
         </is>
       </c>
       <c r="L36" s="2" t="b">
@@ -3522,27 +3714,29 @@
         <v>0</v>
       </c>
       <c r="N36" s="3" t="inlineStr"/>
-      <c r="O36" s="3" t="inlineStr">
-        <is>
-          <t>wrong value: 5 rows returned, ground truth has 4</t>
-        </is>
-      </c>
-      <c r="P36" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q36" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R36" s="2" t="n">
+      <c r="O36" s="3" t="inlineStr"/>
+      <c r="P36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R36" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S36" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T36" s="2" t="n">
         <v>0.000321</v>
       </c>
-      <c r="S36" s="2" t="n">
+      <c r="U36" s="2" t="n">
         <v>0.000113</v>
       </c>
-      <c r="T36" s="2" t="n">
+      <c r="V36" s="2" t="n">
         <v>1.96</v>
       </c>
-      <c r="U36" s="2" t="n">
+      <c r="W36" s="2" t="n">
         <v>1.72</v>
       </c>
     </row>
@@ -3612,22 +3806,28 @@
         </is>
       </c>
       <c r="O37" s="3" t="inlineStr"/>
-      <c r="P37" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q37" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R37" s="2" t="n">
+      <c r="P37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S37" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T37" s="2" t="n">
         <v>0.000432</v>
       </c>
-      <c r="S37" s="2" t="n">
+      <c r="U37" s="2" t="n">
         <v>0.0001</v>
       </c>
-      <c r="T37" s="2" t="n">
+      <c r="V37" s="2" t="n">
         <v>1.91</v>
       </c>
-      <c r="U37" s="2" t="n">
+      <c r="W37" s="2" t="n">
         <v>1.61</v>
       </c>
     </row>
@@ -3674,8 +3874,8 @@
       <c r="H38" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="I38" s="5" t="b">
-        <v>0</v>
+      <c r="I38" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
@@ -3684,7 +3884,7 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>wrong_answer</t>
+          <t>correct</t>
         </is>
       </c>
       <c r="L38" s="2" t="b">
@@ -3694,27 +3894,29 @@
         <v>0</v>
       </c>
       <c r="N38" s="3" t="inlineStr"/>
-      <c r="O38" s="3" t="inlineStr">
-        <is>
-          <t>wrong value: 3 rows returned, ground truth has 2</t>
-        </is>
-      </c>
-      <c r="P38" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q38" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R38" s="2" t="n">
+      <c r="O38" s="3" t="inlineStr"/>
+      <c r="P38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q38" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R38" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S38" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T38" s="2" t="n">
         <v>0.000295</v>
       </c>
-      <c r="S38" s="2" t="n">
+      <c r="U38" s="2" t="n">
         <v>7.8e-05</v>
       </c>
-      <c r="T38" s="2" t="n">
+      <c r="V38" s="2" t="n">
         <v>2.53</v>
       </c>
-      <c r="U38" s="2" t="n">
+      <c r="W38" s="2" t="n">
         <v>1.75</v>
       </c>
     </row>
@@ -3783,22 +3985,28 @@
           <t>answered a question that has no single-table answer (should have been refused)</t>
         </is>
       </c>
-      <c r="P39" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q39" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R39" s="2" t="n">
+      <c r="P39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R39" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S39" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T39" s="2" t="n">
         <v>0.000297</v>
       </c>
-      <c r="S39" s="2" t="n">
+      <c r="U39" s="2" t="n">
         <v>8.6e-05</v>
       </c>
-      <c r="T39" s="2" t="n">
+      <c r="V39" s="2" t="n">
         <v>1.25</v>
       </c>
-      <c r="U39" s="2" t="n">
+      <c r="W39" s="2" t="n">
         <v>1.74</v>
       </c>
     </row>
@@ -3862,22 +4070,28 @@
       </c>
       <c r="N40" s="3" t="inlineStr"/>
       <c r="O40" s="3" t="inlineStr"/>
-      <c r="P40" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q40" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R40" s="2" t="n">
+      <c r="P40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R40" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S40" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T40" s="2" t="n">
         <v>0.0003</v>
       </c>
-      <c r="S40" s="2" t="n">
+      <c r="U40" s="2" t="n">
         <v>9.000000000000001e-05</v>
       </c>
-      <c r="T40" s="2" t="n">
+      <c r="V40" s="2" t="n">
         <v>1.36</v>
       </c>
-      <c r="U40" s="2" t="n">
+      <c r="W40" s="2" t="n">
         <v>4.37</v>
       </c>
     </row>
@@ -3945,22 +4159,28 @@
           <t>answered a question that has no single-table answer (should have been refused)</t>
         </is>
       </c>
-      <c r="P41" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q41" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R41" s="2" t="n">
+      <c r="P41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R41" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S41" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T41" s="2" t="n">
         <v>0.00029</v>
       </c>
-      <c r="S41" s="2" t="n">
+      <c r="U41" s="2" t="n">
         <v>9.899999999999999e-05</v>
       </c>
-      <c r="T41" s="2" t="n">
+      <c r="V41" s="2" t="n">
         <v>1.28</v>
       </c>
-      <c r="U41" s="2" t="n">
+      <c r="W41" s="2" t="n">
         <v>2.31</v>
       </c>
     </row>
@@ -4042,22 +4262,28 @@
           <t>answered a question that has no single-table answer (should have been refused)</t>
         </is>
       </c>
-      <c r="P42" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q42" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R42" s="2" t="n">
+      <c r="P42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R42" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S42" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T42" s="2" t="n">
         <v>0.000579</v>
       </c>
-      <c r="S42" s="2" t="n">
+      <c r="U42" s="2" t="n">
         <v>0.000108</v>
       </c>
-      <c r="T42" s="2" t="n">
+      <c r="V42" s="2" t="n">
         <v>2.8</v>
       </c>
-      <c r="U42" s="2" t="n">
+      <c r="W42" s="2" t="n">
         <v>1.97</v>
       </c>
     </row>
@@ -4139,22 +4365,28 @@
           <t>answered a question that has no single-table answer (should have been refused)</t>
         </is>
       </c>
-      <c r="P43" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q43" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R43" s="2" t="n">
+      <c r="P43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R43" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S43" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T43" s="2" t="n">
         <v>0.000485</v>
       </c>
-      <c r="S43" s="2" t="n">
+      <c r="U43" s="2" t="n">
         <v>0.000149</v>
       </c>
-      <c r="T43" s="2" t="n">
+      <c r="V43" s="2" t="n">
         <v>2.77</v>
       </c>
-      <c r="U43" s="2" t="n">
+      <c r="W43" s="2" t="n">
         <v>1.92</v>
       </c>
     </row>
@@ -4236,22 +4468,28 @@
           <t>answered a question that has no single-table answer (should have been refused)</t>
         </is>
       </c>
-      <c r="P44" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q44" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R44" s="2" t="n">
+      <c r="P44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R44" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S44" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T44" s="2" t="n">
         <v>0.000328</v>
       </c>
-      <c r="S44" s="2" t="n">
+      <c r="U44" s="2" t="n">
         <v>8.2e-05</v>
       </c>
-      <c r="T44" s="2" t="n">
+      <c r="V44" s="2" t="n">
         <v>2.33</v>
       </c>
-      <c r="U44" s="2" t="n">
+      <c r="W44" s="2" t="n">
         <v>1.55</v>
       </c>
     </row>
@@ -4315,22 +4553,28 @@
       </c>
       <c r="N45" s="3" t="inlineStr"/>
       <c r="O45" s="3" t="inlineStr"/>
-      <c r="P45" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q45" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R45" s="2" t="n">
+      <c r="P45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R45" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S45" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T45" s="2" t="n">
         <v>0.000262</v>
       </c>
-      <c r="S45" s="2" t="n">
+      <c r="U45" s="2" t="n">
         <v>8.500000000000001e-05</v>
       </c>
-      <c r="T45" s="2" t="n">
+      <c r="V45" s="2" t="n">
         <v>1.16</v>
       </c>
-      <c r="U45" s="2" t="n">
+      <c r="W45" s="2" t="n">
         <v>0.48</v>
       </c>
     </row>
@@ -4403,22 +4647,28 @@
           <t>answered a question that has no single-table answer (should have been refused)</t>
         </is>
       </c>
-      <c r="P46" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q46" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R46" s="2" t="n">
+      <c r="P46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R46" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S46" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T46" s="2" t="n">
         <v>0.00035</v>
       </c>
-      <c r="S46" s="2" t="n">
+      <c r="U46" s="2" t="n">
         <v>9.6e-05</v>
       </c>
-      <c r="T46" s="2" t="n">
+      <c r="V46" s="2" t="n">
         <v>2.34</v>
       </c>
-      <c r="U46" s="2" t="n">
+      <c r="W46" s="2" t="n">
         <v>1.87</v>
       </c>
     </row>
@@ -4490,22 +4740,28 @@
           <t>[error] error: AttributeError: 'DataFrame' object has no attribute 'to_frame'</t>
         </is>
       </c>
-      <c r="P47" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q47" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R47" s="2" t="n">
+      <c r="P47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R47" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S47" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T47" s="2" t="n">
         <v>0.000329</v>
       </c>
-      <c r="S47" s="2" t="n">
+      <c r="U47" s="2" t="n">
         <v>9.3e-05</v>
       </c>
-      <c r="T47" s="2" t="n">
+      <c r="V47" s="2" t="n">
         <v>3.02</v>
       </c>
-      <c r="U47" s="2" t="n">
+      <c r="W47" s="2" t="n">
         <v>1.67</v>
       </c>
     </row>
@@ -4573,22 +4829,28 @@
           <t>answered a question that has no single-table answer (should have been refused)</t>
         </is>
       </c>
-      <c r="P48" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q48" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R48" s="2" t="n">
+      <c r="P48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R48" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S48" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T48" s="2" t="n">
         <v>0.000433</v>
       </c>
-      <c r="S48" s="2" t="n">
+      <c r="U48" s="2" t="n">
         <v>0.000111</v>
       </c>
-      <c r="T48" s="2" t="n">
+      <c r="V48" s="2" t="n">
         <v>3.41</v>
       </c>
-      <c r="U48" s="2" t="n">
+      <c r="W48" s="2" t="n">
         <v>1.75</v>
       </c>
     </row>
@@ -4652,22 +4914,28 @@
       </c>
       <c r="N49" s="3" t="inlineStr"/>
       <c r="O49" s="3" t="inlineStr"/>
-      <c r="P49" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q49" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R49" s="2" t="n">
+      <c r="P49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R49" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S49" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T49" s="2" t="n">
         <v>0.0005910000000000001</v>
       </c>
-      <c r="S49" s="2" t="n">
+      <c r="U49" s="2" t="n">
         <v>0.000169</v>
       </c>
-      <c r="T49" s="2" t="n">
+      <c r="V49" s="2" t="n">
         <v>7.58</v>
       </c>
-      <c r="U49" s="2" t="n">
+      <c r="W49" s="2" t="n">
         <v>3.12</v>
       </c>
     </row>
@@ -4731,22 +4999,28 @@
       </c>
       <c r="N50" s="3" t="inlineStr"/>
       <c r="O50" s="3" t="inlineStr"/>
-      <c r="P50" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q50" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R50" s="2" t="n">
+      <c r="P50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R50" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S50" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T50" s="2" t="n">
         <v>0.000899</v>
       </c>
-      <c r="S50" s="2" t="n">
+      <c r="U50" s="2" t="n">
         <v>0.000258</v>
       </c>
-      <c r="T50" s="2" t="n">
+      <c r="V50" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="U50" s="2" t="n">
+      <c r="W50" s="2" t="n">
         <v>5.36</v>
       </c>
     </row>
@@ -4814,22 +5088,28 @@
         </is>
       </c>
       <c r="O51" s="3" t="inlineStr"/>
-      <c r="P51" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q51" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R51" s="2" t="n">
+      <c r="P51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R51" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S51" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T51" s="2" t="n">
         <v>0.000555</v>
       </c>
-      <c r="S51" s="2" t="n">
+      <c r="U51" s="2" t="n">
         <v>0.000164</v>
       </c>
-      <c r="T51" s="2" t="n">
+      <c r="V51" s="2" t="n">
         <v>4.58</v>
       </c>
-      <c r="U51" s="2" t="n">
+      <c r="W51" s="2" t="n">
         <v>3.2</v>
       </c>
     </row>
@@ -4897,22 +5177,28 @@
         </is>
       </c>
       <c r="O52" s="3" t="inlineStr"/>
-      <c r="P52" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q52" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R52" s="2" t="n">
+      <c r="P52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R52" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S52" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T52" s="2" t="n">
         <v>0.00083</v>
       </c>
-      <c r="S52" s="2" t="n">
+      <c r="U52" s="2" t="n">
         <v>0.000251</v>
       </c>
-      <c r="T52" s="2" t="n">
+      <c r="V52" s="2" t="n">
         <v>6.9</v>
       </c>
-      <c r="U52" s="2" t="n">
+      <c r="W52" s="2" t="n">
         <v>4.81</v>
       </c>
     </row>
@@ -4976,22 +5262,28 @@
       </c>
       <c r="N53" s="3" t="inlineStr"/>
       <c r="O53" s="3" t="inlineStr"/>
-      <c r="P53" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q53" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R53" s="2" t="n">
+      <c r="P53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R53" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S53" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T53" s="2" t="n">
         <v>0.000579</v>
       </c>
-      <c r="S53" s="2" t="n">
+      <c r="U53" s="2" t="n">
         <v>0.000166</v>
       </c>
-      <c r="T53" s="2" t="n">
+      <c r="V53" s="2" t="n">
         <v>5.05</v>
       </c>
-      <c r="U53" s="2" t="n">
+      <c r="W53" s="2" t="n">
         <v>3.22</v>
       </c>
     </row>
@@ -5055,22 +5347,28 @@
       </c>
       <c r="N54" s="3" t="inlineStr"/>
       <c r="O54" s="3" t="inlineStr"/>
-      <c r="P54" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q54" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R54" s="2" t="n">
+      <c r="P54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R54" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S54" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T54" s="2" t="n">
         <v>0.000871</v>
       </c>
-      <c r="S54" s="2" t="n">
+      <c r="U54" s="2" t="n">
         <v>0.000252</v>
       </c>
-      <c r="T54" s="2" t="n">
+      <c r="V54" s="2" t="n">
         <v>6.91</v>
       </c>
-      <c r="U54" s="2" t="n">
+      <c r="W54" s="2" t="n">
         <v>4.65</v>
       </c>
     </row>
@@ -5134,22 +5432,28 @@
         </is>
       </c>
       <c r="O55" s="3" t="inlineStr"/>
-      <c r="P55" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q55" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R55" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S55" s="2" t="n">
+      <c r="P55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R55" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S55" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U55" s="2" t="n">
         <v>0.000168</v>
       </c>
-      <c r="T55" s="2" t="n">
+      <c r="V55" s="2" t="n">
         <v>2.63</v>
       </c>
-      <c r="U55" s="2" t="n">
+      <c r="W55" s="2" t="n">
         <v>3.15</v>
       </c>
     </row>
@@ -5213,22 +5517,28 @@
       </c>
       <c r="N56" s="3" t="inlineStr"/>
       <c r="O56" s="3" t="inlineStr"/>
-      <c r="P56" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q56" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R56" s="2" t="n">
+      <c r="P56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R56" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S56" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T56" s="2" t="n">
         <v>0.000837</v>
       </c>
-      <c r="S56" s="2" t="n">
+      <c r="U56" s="2" t="n">
         <v>0.000245</v>
       </c>
-      <c r="T56" s="2" t="n">
+      <c r="V56" s="2" t="n">
         <v>7.83</v>
       </c>
-      <c r="U56" s="2" t="n">
+      <c r="W56" s="2" t="n">
         <v>4.71</v>
       </c>
     </row>
@@ -5301,22 +5611,28 @@
           <t>wrong value: 273 rows returned, ground truth has 1</t>
         </is>
       </c>
-      <c r="P57" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q57" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R57" s="2" t="n">
+      <c r="P57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R57" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S57" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T57" s="2" t="n">
         <v>0.00066</v>
       </c>
-      <c r="S57" s="2" t="n">
+      <c r="U57" s="2" t="n">
         <v>0.000187</v>
       </c>
-      <c r="T57" s="2" t="n">
+      <c r="V57" s="2" t="n">
         <v>8.369999999999999</v>
       </c>
-      <c r="U57" s="2" t="n">
+      <c r="W57" s="2" t="n">
         <v>3.3</v>
       </c>
     </row>
@@ -5380,22 +5696,28 @@
       </c>
       <c r="N58" s="3" t="inlineStr"/>
       <c r="O58" s="3" t="inlineStr"/>
-      <c r="P58" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q58" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R58" s="2" t="n">
+      <c r="P58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R58" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S58" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T58" s="2" t="n">
         <v>0.000971</v>
       </c>
-      <c r="S58" s="2" t="n">
+      <c r="U58" s="2" t="n">
         <v>0.000276</v>
       </c>
-      <c r="T58" s="2" t="n">
+      <c r="V58" s="2" t="n">
         <v>11.34</v>
       </c>
-      <c r="U58" s="2" t="n">
+      <c r="W58" s="2" t="n">
         <v>4.78</v>
       </c>
     </row>
@@ -5459,22 +5781,28 @@
       </c>
       <c r="N59" s="3" t="inlineStr"/>
       <c r="O59" s="3" t="inlineStr"/>
-      <c r="P59" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q59" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R59" s="2" t="n">
+      <c r="P59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R59" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S59" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T59" s="2" t="n">
         <v>0.000576</v>
       </c>
-      <c r="S59" s="2" t="n">
+      <c r="U59" s="2" t="n">
         <v>0.000177</v>
       </c>
-      <c r="T59" s="2" t="n">
+      <c r="V59" s="2" t="n">
         <v>4.28</v>
       </c>
-      <c r="U59" s="2" t="n">
+      <c r="W59" s="2" t="n">
         <v>3.89</v>
       </c>
     </row>
@@ -5538,22 +5866,28 @@
       </c>
       <c r="N60" s="3" t="inlineStr"/>
       <c r="O60" s="3" t="inlineStr"/>
-      <c r="P60" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q60" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R60" s="2" t="n">
+      <c r="P60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R60" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S60" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T60" s="2" t="n">
         <v>0.000856</v>
       </c>
-      <c r="S60" s="2" t="n">
+      <c r="U60" s="2" t="n">
         <v>0.000267</v>
       </c>
-      <c r="T60" s="2" t="n">
+      <c r="V60" s="2" t="n">
         <v>6.64</v>
       </c>
-      <c r="U60" s="2" t="n">
+      <c r="W60" s="2" t="n">
         <v>5.23</v>
       </c>
     </row>
@@ -5621,22 +5955,28 @@
         </is>
       </c>
       <c r="O61" s="3" t="inlineStr"/>
-      <c r="P61" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q61" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R61" s="2" t="n">
+      <c r="P61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R61" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S61" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T61" s="2" t="n">
         <v>0.001458</v>
       </c>
-      <c r="S61" s="2" t="n">
+      <c r="U61" s="2" t="n">
         <v>0.000376</v>
       </c>
-      <c r="T61" s="2" t="n">
+      <c r="V61" s="2" t="n">
         <v>17.3</v>
       </c>
-      <c r="U61" s="2" t="n">
+      <c r="W61" s="2" t="n">
         <v>6.69</v>
       </c>
     </row>
@@ -5704,22 +6044,28 @@
           <t>wrong value: row 1: 719,047.03 vs 122,490.80</t>
         </is>
       </c>
-      <c r="P62" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q62" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R62" s="2" t="n">
+      <c r="P62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R62" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S62" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T62" s="2" t="n">
         <v>0.001133</v>
       </c>
-      <c r="S62" s="2" t="n">
+      <c r="U62" s="2" t="n">
         <v>0.000341</v>
       </c>
-      <c r="T62" s="2" t="n">
+      <c r="V62" s="2" t="n">
         <v>8.710000000000001</v>
       </c>
-      <c r="U62" s="2" t="n">
+      <c r="W62" s="2" t="n">
         <v>6.38</v>
       </c>
     </row>
@@ -5794,22 +6140,28 @@
         </is>
       </c>
       <c r="O63" s="3" t="inlineStr"/>
-      <c r="P63" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q63" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R63" s="2" t="n">
+      <c r="P63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q63" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R63" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S63" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T63" s="2" t="n">
         <v>0.002317</v>
       </c>
-      <c r="S63" s="2" t="n">
+      <c r="U63" s="2" t="n">
         <v>0.000362</v>
       </c>
-      <c r="T63" s="2" t="n">
+      <c r="V63" s="2" t="n">
         <v>20.51</v>
       </c>
-      <c r="U63" s="2" t="n">
+      <c r="W63" s="2" t="n">
         <v>6.62</v>
       </c>
     </row>
@@ -5856,15 +6208,15 @@
 Region=West | Profit=108,418.45</t>
         </is>
       </c>
-      <c r="H64" s="5" t="b">
-        <v>0</v>
+      <c r="H64" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="I64" s="4" t="b">
         <v>1</v>
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>wrong_answer</t>
+          <t>correct</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
@@ -5878,33 +6230,35 @@
       <c r="M64" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="N64" s="3" t="inlineStr">
-        <is>
-          <t>Planner: superset result (extra rows) | wrong value: 4 rows returned, ground truth has 3</t>
-        </is>
-      </c>
+      <c r="N64" s="3" t="inlineStr"/>
       <c r="O64" s="3" t="inlineStr"/>
-      <c r="P64" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q64" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="R64" s="2" t="n">
+      <c r="P64" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R64" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S64" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T64" s="2" t="n">
         <v>0.001092</v>
       </c>
-      <c r="S64" s="2" t="n">
+      <c r="U64" s="2" t="n">
         <v>0.000338</v>
       </c>
-      <c r="T64" s="2" t="n">
+      <c r="V64" s="2" t="n">
         <v>8.279999999999999</v>
       </c>
-      <c r="U64" s="2" t="n">
+      <c r="W64" s="2" t="n">
         <v>6.4</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U64"/>
+  <autoFilter ref="A1:W64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5915,7 +6269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -5927,7 +6281,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Matches ground truth (column names ignored): of all 63 queries and of the 53 answerable ones</t>
+          <t>Matches ground truth (column names ignored, extra rows allowed): of all 63 queries and of the 53 answerable ones</t>
         </is>
       </c>
     </row>
@@ -5951,10 +6305,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C3" t="n">
-        <v>41</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4">
@@ -5964,10 +6318,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C4" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5">
@@ -5986,207 +6340,210 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>All 63 under STRICT scoring (column names must match)</t>
+          <t xml:space="preserve">  of which correct only because extra rows are allowed</t>
         </is>
       </c>
       <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>All 63 under STRICT scoring (column names and row count must match)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>48</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C7" t="n">
         <v>36</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Outcome counts, answerable queries only</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>outcome</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>ADAA</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>Code-writing system</t>
         </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>correct</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>43</v>
-      </c>
-      <c r="C10" t="n">
-        <v>39</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>wrong_answer</t>
+          <t>correct</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="C11" t="n">
-        <v>13</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>wrong_answer</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>refused_correctly</t>
+          <t>error</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>refused_correctly</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>refused_wrongly</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B15" t="n">
         <v>2</v>
       </c>
-      <c r="C14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Outcome counts, compound queries (correct = refuse), 10 queries</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>outcome</t>
         </is>
       </c>
-      <c r="B17" s="1" t="inlineStr">
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>ADAA</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>Code-writing system</t>
         </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>refused_correctly</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>5</v>
-      </c>
-      <c r="C18" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>answered_should_refuse</t>
+          <t>refused_correctly</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>answered_should_refuse</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>5</v>
+      </c>
+      <c r="C20" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>error</t>
         </is>
       </c>
-      <c r="B20" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="B21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Who is right where (all queries)</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr"/>
-      <c r="B23" s="1" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr"/>
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>queries</t>
         </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>both correct</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>32</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>only ADAA correct</t>
+          <t>both correct</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>only code system correct</t>
+          <t>only ADAA correct</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -6196,69 +6553,63 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>only code system correct</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>both not correct</t>
         </is>
       </c>
-      <c r="B27" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
+      <c r="B28" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>By category</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="B30" s="1" t="inlineStr">
+      <c r="B31" s="1" t="inlineStr">
         <is>
           <t>queries</t>
         </is>
       </c>
-      <c r="C30" s="1" t="inlineStr">
+      <c r="C31" s="1" t="inlineStr">
         <is>
           <t>ADAA correct</t>
         </is>
       </c>
-      <c r="D30" s="1" t="inlineStr">
+      <c r="D31" s="1" t="inlineStr">
         <is>
           <t>Code system correct</t>
         </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>1. Simple aggregation</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>5</v>
-      </c>
-      <c r="C31" t="n">
-        <v>5</v>
-      </c>
-      <c r="D31" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2. Filtering</t>
+          <t>1. Simple aggregation</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>5</v>
       </c>
       <c r="C32" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D32" t="n">
         <v>5</v>
@@ -6267,23 +6618,23 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>3. Grouping + ranking</t>
+          <t>2. Filtering</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>5</v>
       </c>
       <c r="C33" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" t="n">
         <v>5</v>
-      </c>
-      <c r="D33" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>4. Time based</t>
+          <t>3. Grouping + ranking</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -6293,13 +6644,13 @@
         <v>5</v>
       </c>
       <c r="D34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>5. Multi-condition</t>
+          <t>4. Time based</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -6309,13 +6660,13 @@
         <v>5</v>
       </c>
       <c r="D35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>6. Derived calculations</t>
+          <t>5. Multi-condition</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -6325,68 +6676,68 @@
         <v>5</v>
       </c>
       <c r="D36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>7. Pseudo-compound: breakdown</t>
+          <t>6. Derived calculations</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>5</v>
       </c>
       <c r="C37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D37" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>7. Pseudo-compound: comparison</t>
+          <t>7. Pseudo-compound: breakdown</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>8. Compound: filter + two aggregates</t>
+          <t>7. Pseudo-compound: comparison</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C39" t="n">
         <v>1</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>8. Compound: scalar + ranked list</t>
+          <t>8. Compound: filter + two aggregates</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
@@ -6395,30 +6746,30 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>8. Compound: two grouped outputs</t>
+          <t>8. Compound: scalar + ranked list</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>8. Compound: two scalars</t>
+          <t>8. Compound: two grouped outputs</t>
         </is>
       </c>
       <c r="B42" t="n">
         <v>3</v>
       </c>
       <c r="C42" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D42" t="n">
         <v>1</v>
@@ -6427,159 +6778,175 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>9. Multi-turn (2 turns)</t>
+          <t>8. Compound: two scalars</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D43" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>9. Multi-turn (3 turns)</t>
+          <t>9. Multi-turn (2 turns)</t>
         </is>
       </c>
       <c r="B44" t="n">
         <v>6</v>
       </c>
       <c r="C44" t="n">
+        <v>4</v>
+      </c>
+      <c r="D44" t="n">
         <v>5</v>
-      </c>
-      <c r="D44" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>9. Multi-turn (3 turns)</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>6</v>
+      </c>
+      <c r="C45" t="n">
+        <v>5</v>
+      </c>
+      <c r="D45" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>9. Multi-turn (4 turns)</t>
         </is>
       </c>
-      <c r="B45" t="n">
+      <c r="B46" t="n">
         <v>4</v>
       </c>
-      <c r="C45" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" t="n">
+      <c r="C46" t="n">
+        <v>2</v>
+      </c>
+      <c r="D46" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="6" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>Cost and time</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="1" t="inlineStr"/>
-      <c r="B48" s="1" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr"/>
+      <c r="B49" s="1" t="inlineStr">
         <is>
           <t>ADAA</t>
         </is>
       </c>
-      <c r="C48" s="1" t="inlineStr">
+      <c r="C49" s="1" t="inlineStr">
         <is>
           <t>Code-writing system</t>
         </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>total cost (USD)</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>0.0292</v>
-      </c>
-      <c r="C49" t="n">
-        <v>0.008410000000000001</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>cost per query (USD)</t>
+          <t>total cost (USD)</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0.00046</v>
+        <v>0.0292</v>
       </c>
       <c r="C50" t="n">
-        <v>0.00013</v>
+        <v>0.008410000000000001</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>total time (s)</t>
+          <t>cost per query (USD)</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>263</v>
+        <v>0.00046</v>
       </c>
       <c r="C51" t="n">
-        <v>159</v>
+        <v>0.00013</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>time per query (s)</t>
+          <t>total time (s)</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>4.2</v>
+        <v>263</v>
       </c>
       <c r="C52" t="n">
-        <v>2.5</v>
+        <v>159</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>input tokens</t>
+          <t>time per query (s)</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>285439</v>
+        <v>4.2</v>
       </c>
       <c r="C53" t="n">
-        <v>84528</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>output tokens</t>
+          <t>input tokens</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>25975</v>
+        <v>285439</v>
       </c>
       <c r="C54" t="n">
-        <v>6896</v>
+        <v>84528</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>output tokens</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>25975</v>
+      </c>
+      <c r="C55" t="n">
+        <v>6896</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>LLM calls</t>
         </is>
       </c>
-      <c r="B55" t="n">
+      <c r="B56" t="n">
         <v>183</v>
       </c>
-      <c r="C55" t="n">
+      <c r="C56" t="n">
         <v>93</v>
       </c>
     </row>
@@ -6594,7 +6961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -6658,85 +7025,92 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>gt_vs_adaa / gt_vs_llm: TRUE when the system's table matches ground truth. Values and row order are compared with 1% relative tolerance; column names and column order are ignored. For the 10 compound queries (Q38-Q47, no ground truth) TRUE means the system refused.</t>
+          <t>gt_vs_adaa / gt_vs_llm: TRUE when every ground-truth row is present in the system's table (1% relative tolerance). EXTRA ROWS ARE ALLOWED (for example 4 correct region rows plus a Total row is correct; decided by the user, applied to both systems). Column names and column order are ignored; row order must be kept for ranked questions. For the 10 compound queries (Q38-Q47, no ground truth) TRUE means the system refused.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>adaa_error / llm_error: TRUE only when the system produced NO usable answer (crash, blocked by the sandbox, tool error, skipped).</t>
+          <t>adaa_extra_rows / llm_extra_rows: how many rows beyond ground truth a correct answer contained (0 if none).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>A WRONG ANSWER is not an error: it has error = FALSE, match = FALSE and outcome = wrong_answer. A wrong refusal is not an error either (outcome = refused_wrongly).</t>
+          <t>adaa_error / llm_error: TRUE only when the system produced NO usable answer (crash, blocked by the sandbox, tool error, skipped).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>outcome values: correct, wrong_answer, error, refused_correctly, refused_wrongly, answered_should_refuse.</t>
+          <t>A WRONG ANSWER is not an error: it has error = FALSE, match = FALSE and outcome = wrong_answer. A wrong refusal is not an error either (outcome = refused_wrongly).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>adaa_error_reason: ADAA's Part C failure category (from the failure-cause labeller) plus the detail. llm_error_reason: sandbox status and message, or the first differing value, or the refusal.</t>
+          <t>outcome values: correct, wrong_answer, error, refused_correctly, refused_wrongly, answered_should_refuse.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>adaa_strict_match / llm_strict_match: the original harness score, where column names must also match. Kept for transparency.</t>
+          <t>adaa_error_reason: ADAA's Part C failure category (from the failure-cause labeller) plus the detail. llm_error_reason: sandbox status and message, or the first differing value, or the refusal.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr"/>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>adaa_strict_match / llm_strict_match: the original harness score, where column names and the row count must also match. Kept for transparency.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>CAVEATS</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>One run per system: ADAA varies run to run (see the B3 consistency findings in docs/v2-polish-plan.md), so small differences are not significant.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>ADAA's cost and time include an answer-writing LLM call and a larger planner prompt; the code-writing system returns a table only, with no sentence.</t>
+          <t>One run per system: ADAA varies run to run (see the B3 consistency findings in docs/v2-polish-plan.md), so small differences are not significant.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>The code-writing system's sandbox is a restricted exec, adequate for this experiment on a public dataset but not safe for untrusted users.</t>
+          <t>ADAA's cost and time include an answer-writing LLM call and a larger planner prompt; the code-writing system returns a table only, with no sentence.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>The code system was given the same one-table contract and an explicit REFUSE option as ADAA's planner has (prompt version v2).</t>
+          <t>The code-writing system's sandbox is a restricted exec, adequate for this experiment on a public dataset but not safe for untrusted users.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>The code system was given the same one-table contract and an explicit REFUSE option as ADAA's planner has (prompt version v2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>The sandbox allows only plainly safe df.query strings; anything else on its deny list is blocked and counts as an error.</t>
         </is>

</xml_diff>